<commit_message>
Put the grade band label in a single cell
The band header split GRADE 1 and 12 topics across two cells on the
same navy bar, so it ran together and read as GRADE 1 12. It is now
one string in the topic column, GRADE 1 with a middot and 12 topics,
with the grade column left empty on band rows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CpNuKcjfG2EQrbJ8Wsoe9D
</commit_message>
<xml_diff>
--- a/tutoring/charlotte/Charlotte_RAG_mathsgenie.xlsx
+++ b/tutoring/charlotte/Charlotte_RAG_mathsgenie.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="239">
   <si>
     <t xml:space="preserve">Summary</t>
   </si>
@@ -180,10 +180,7 @@
     <t xml:space="preserve">Ans</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 topics</t>
+    <t xml:space="preserve">GRADE 1   ·   12 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Addition And Subtraction</t>
@@ -246,10 +243,7 @@
     <t xml:space="preserve">Interpreting Data</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 topics</t>
+    <t xml:space="preserve">GRADE 2   ·   16 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Calculation Problems</t>
@@ -327,10 +321,7 @@
     <t xml:space="preserve">Pie Charts</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18 topics</t>
+    <t xml:space="preserve">GRADE 3   ·   18 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Estimating</t>
@@ -411,7 +402,7 @@
     <t xml:space="preserve">Frequency Trees</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 4</t>
+    <t xml:space="preserve">GRADE 4   ·   18 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Compound Interest And Depreciation</t>
@@ -492,10 +483,7 @@
     <t xml:space="preserve">Frequency Tables</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 topics</t>
+    <t xml:space="preserve">GRADE 5   ·   13 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Reverse Percentages</t>
@@ -561,10 +549,7 @@
     <t xml:space="preserve">Data</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17 topics</t>
+    <t xml:space="preserve">GRADE 6   ·   17 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Recurring Decimals To Fractions</t>
@@ -651,10 +636,7 @@
     <t xml:space="preserve">Tree Diagrams</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 topics</t>
+    <t xml:space="preserve">GRADE 7   ·   15 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Surds</t>
@@ -708,10 +690,7 @@
     <t xml:space="preserve">Conditional Probability</t>
   </si>
   <si>
-    <t xml:space="preserve">GRADE 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 topics</t>
+    <t xml:space="preserve">GRADE 8   ·   10 topics</t>
   </si>
   <si>
     <t xml:space="preserve">Quadratic Simultaneous Equations</t>
@@ -1962,12 +1941,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="19"/>
+      <c r="B2" s="20" t="s">
         <v>52</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>53</v>
       </c>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
@@ -1982,15 +1959,15 @@
         <v>1</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="24"/>
       <c r="E3" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="G3" s="25" t="s">
         <v>49</v>
@@ -2007,15 +1984,15 @@
         <v>1</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="24"/>
       <c r="E4" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="G4" s="25" t="s">
         <v>49</v>
@@ -2032,15 +2009,15 @@
         <v>1</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="24"/>
       <c r="E5" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G5" s="25" t="s">
         <v>49</v>
@@ -2057,15 +2034,15 @@
         <v>1</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="24"/>
       <c r="E6" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G6" s="25" t="s">
         <v>49</v>
@@ -2082,15 +2059,15 @@
         <v>1</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="24"/>
       <c r="E7" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G7" s="26"/>
       <c r="H7" s="26"/>
@@ -2101,15 +2078,15 @@
         <v>1</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" s="23"/>
       <c r="D8" s="24"/>
       <c r="E8" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G8" s="25" t="s">
         <v>49</v>
@@ -2126,15 +2103,15 @@
         <v>1</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C9" s="23"/>
       <c r="D9" s="24"/>
       <c r="E9" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="G9" s="25" t="s">
         <v>49</v>
@@ -2151,15 +2128,15 @@
         <v>1</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="23"/>
       <c r="D10" s="24"/>
       <c r="E10" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G10" s="25" t="s">
         <v>49</v>
@@ -2176,15 +2153,15 @@
         <v>1</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C11" s="23"/>
       <c r="D11" s="24"/>
       <c r="E11" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="G11" s="25" t="s">
         <v>49</v>
@@ -2201,15 +2178,15 @@
         <v>1</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C12" s="23"/>
       <c r="D12" s="24"/>
       <c r="E12" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G12" s="25" t="s">
         <v>49</v>
@@ -2226,15 +2203,15 @@
         <v>1</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C13" s="23"/>
       <c r="D13" s="24"/>
       <c r="E13" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G13" s="25" t="s">
         <v>49</v>
@@ -2251,32 +2228,30 @@
         <v>1</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="24"/>
       <c r="E14" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F14" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="H14" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="I14" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19"/>
+      <c r="B15" s="20" t="s">
         <v>73</v>
-      </c>
-      <c r="G14" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="H14" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="I14" s="25" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>75</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
@@ -2291,15 +2266,15 @@
         <v>2</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="24"/>
       <c r="E16" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G16" s="25" t="s">
         <v>49</v>
@@ -2316,15 +2291,15 @@
         <v>2</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="24"/>
       <c r="E17" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G17" s="26"/>
       <c r="H17" s="26"/>
@@ -2335,15 +2310,15 @@
         <v>2</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="24"/>
       <c r="E18" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G18" s="25" t="s">
         <v>49</v>
@@ -2360,15 +2335,15 @@
         <v>2</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="24"/>
       <c r="E19" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G19" s="25" t="s">
         <v>49</v>
@@ -2385,15 +2360,15 @@
         <v>2</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="24"/>
       <c r="E20" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G20" s="25" t="s">
         <v>49</v>
@@ -2410,15 +2385,15 @@
         <v>2</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C21" s="23"/>
       <c r="D21" s="24"/>
       <c r="E21" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G21" s="25" t="s">
         <v>49</v>
@@ -2435,15 +2410,15 @@
         <v>2</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C22" s="23"/>
       <c r="D22" s="24"/>
       <c r="E22" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G22" s="25" t="s">
         <v>49</v>
@@ -2460,15 +2435,15 @@
         <v>2</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C23" s="23"/>
       <c r="D23" s="24"/>
       <c r="E23" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G23" s="26"/>
       <c r="H23" s="26"/>
@@ -2479,15 +2454,15 @@
         <v>2</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C24" s="23"/>
       <c r="D24" s="24"/>
       <c r="E24" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G24" s="25" t="s">
         <v>49</v>
@@ -2504,15 +2479,15 @@
         <v>2</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C25" s="23"/>
       <c r="D25" s="24"/>
       <c r="E25" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G25" s="25" t="s">
         <v>49</v>
@@ -2529,15 +2504,15 @@
         <v>2</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C26" s="23"/>
       <c r="D26" s="24"/>
       <c r="E26" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G26" s="25" t="s">
         <v>49</v>
@@ -2554,15 +2529,15 @@
         <v>2</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C27" s="23"/>
       <c r="D27" s="24"/>
       <c r="E27" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G27" s="25" t="s">
         <v>49</v>
@@ -2579,15 +2554,15 @@
         <v>2</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C28" s="23"/>
       <c r="D28" s="24"/>
       <c r="E28" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G28" s="25" t="s">
         <v>49</v>
@@ -2604,15 +2579,15 @@
         <v>2</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C29" s="23"/>
       <c r="D29" s="24"/>
       <c r="E29" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G29" s="25" t="s">
         <v>49</v>
@@ -2629,15 +2604,15 @@
         <v>2</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C30" s="23"/>
       <c r="D30" s="24"/>
       <c r="E30" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G30" s="25" t="s">
         <v>49</v>
@@ -2654,15 +2629,15 @@
         <v>2</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C31" s="23"/>
       <c r="D31" s="24"/>
       <c r="E31" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G31" s="25" t="s">
         <v>49</v>
@@ -2674,12 +2649,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
-        <v>101</v>
-      </c>
+    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19"/>
       <c r="B32" s="20" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C32" s="20"/>
       <c r="D32" s="20"/>
@@ -2694,15 +2667,15 @@
         <v>3</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C33" s="23"/>
       <c r="D33" s="24"/>
       <c r="E33" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G33" s="25" t="s">
         <v>49</v>
@@ -2719,15 +2692,15 @@
         <v>3</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C34" s="23"/>
       <c r="D34" s="24"/>
       <c r="E34" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G34" s="25" t="s">
         <v>49</v>
@@ -2744,15 +2717,15 @@
         <v>3</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C35" s="23"/>
       <c r="D35" s="24"/>
       <c r="E35" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G35" s="25" t="s">
         <v>49</v>
@@ -2769,15 +2742,15 @@
         <v>3</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C36" s="23"/>
       <c r="D36" s="24"/>
       <c r="E36" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G36" s="25" t="s">
         <v>49</v>
@@ -2794,15 +2767,15 @@
         <v>3</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C37" s="23"/>
       <c r="D37" s="24"/>
       <c r="E37" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G37" s="25" t="s">
         <v>49</v>
@@ -2819,15 +2792,15 @@
         <v>3</v>
       </c>
       <c r="B38" s="22" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C38" s="23"/>
       <c r="D38" s="24"/>
       <c r="E38" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G38" s="25" t="s">
         <v>49</v>
@@ -2844,15 +2817,15 @@
         <v>3</v>
       </c>
       <c r="B39" s="22" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C39" s="23"/>
       <c r="D39" s="24"/>
       <c r="E39" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F39" s="15" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G39" s="25" t="s">
         <v>49</v>
@@ -2869,15 +2842,15 @@
         <v>3</v>
       </c>
       <c r="B40" s="22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C40" s="23"/>
       <c r="D40" s="24"/>
       <c r="E40" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G40" s="25" t="s">
         <v>49</v>
@@ -2894,15 +2867,15 @@
         <v>3</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C41" s="23"/>
       <c r="D41" s="24"/>
       <c r="E41" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G41" s="25" t="s">
         <v>49</v>
@@ -2919,15 +2892,15 @@
         <v>3</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C42" s="23"/>
       <c r="D42" s="24"/>
       <c r="E42" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G42" s="25" t="s">
         <v>49</v>
@@ -2944,15 +2917,15 @@
         <v>3</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C43" s="23"/>
       <c r="D43" s="24"/>
       <c r="E43" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G43" s="25" t="s">
         <v>49</v>
@@ -2969,15 +2942,15 @@
         <v>3</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C44" s="23"/>
       <c r="D44" s="24"/>
       <c r="E44" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G44" s="25" t="s">
         <v>49</v>
@@ -2994,15 +2967,15 @@
         <v>3</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C45" s="23"/>
       <c r="D45" s="24"/>
       <c r="E45" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F45" s="15" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G45" s="25" t="s">
         <v>49</v>
@@ -3019,15 +2992,15 @@
         <v>3</v>
       </c>
       <c r="B46" s="22" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C46" s="23"/>
       <c r="D46" s="24"/>
       <c r="E46" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G46" s="25" t="s">
         <v>49</v>
@@ -3044,15 +3017,15 @@
         <v>3</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C47" s="23"/>
       <c r="D47" s="24"/>
       <c r="E47" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G47" s="25" t="s">
         <v>49</v>
@@ -3069,15 +3042,15 @@
         <v>3</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C48" s="23"/>
       <c r="D48" s="24"/>
       <c r="E48" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G48" s="25" t="s">
         <v>49</v>
@@ -3094,15 +3067,15 @@
         <v>3</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C49" s="23"/>
       <c r="D49" s="24"/>
       <c r="E49" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F49" s="15" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G49" s="25" t="s">
         <v>49</v>
@@ -3119,15 +3092,15 @@
         <v>3</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C50" s="23"/>
       <c r="D50" s="24"/>
       <c r="E50" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G50" s="25" t="s">
         <v>49</v>
@@ -3139,12 +3112,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="19" t="s">
-        <v>129</v>
-      </c>
+    <row r="51" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="19"/>
       <c r="B51" s="20" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="C51" s="20"/>
       <c r="D51" s="20"/>
@@ -3159,15 +3130,15 @@
         <v>4</v>
       </c>
       <c r="B52" s="28" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C52" s="23"/>
       <c r="D52" s="24"/>
       <c r="E52" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G52" s="25" t="s">
         <v>49</v>
@@ -3189,7 +3160,7 @@
       <c r="C53" s="23"/>
       <c r="D53" s="24"/>
       <c r="E53" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F53" s="15" t="s">
         <v>45</v>
@@ -3209,15 +3180,15 @@
         <v>4</v>
       </c>
       <c r="B54" s="28" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C54" s="23"/>
       <c r="D54" s="24"/>
       <c r="E54" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F54" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G54" s="25" t="s">
         <v>49</v>
@@ -3234,15 +3205,15 @@
         <v>4</v>
       </c>
       <c r="B55" s="28" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C55" s="23"/>
       <c r="D55" s="24"/>
       <c r="E55" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G55" s="25" t="s">
         <v>49</v>
@@ -3259,15 +3230,15 @@
         <v>4</v>
       </c>
       <c r="B56" s="28" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C56" s="23"/>
       <c r="D56" s="24"/>
       <c r="E56" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F56" s="15" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="G56" s="25" t="s">
         <v>49</v>
@@ -3284,15 +3255,15 @@
         <v>4</v>
       </c>
       <c r="B57" s="28" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C57" s="23"/>
       <c r="D57" s="24"/>
       <c r="E57" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F57" s="15" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G57" s="25" t="s">
         <v>49</v>
@@ -3309,15 +3280,15 @@
         <v>4</v>
       </c>
       <c r="B58" s="28" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C58" s="23"/>
       <c r="D58" s="24"/>
       <c r="E58" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F58" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G58" s="25" t="s">
         <v>49</v>
@@ -3334,15 +3305,15 @@
         <v>4</v>
       </c>
       <c r="B59" s="28" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C59" s="23"/>
       <c r="D59" s="24"/>
       <c r="E59" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F59" s="15" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G59" s="25" t="s">
         <v>49</v>
@@ -3359,15 +3330,15 @@
         <v>4</v>
       </c>
       <c r="B60" s="28" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C60" s="23"/>
       <c r="D60" s="24"/>
       <c r="E60" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G60" s="25" t="s">
         <v>49</v>
@@ -3384,15 +3355,15 @@
         <v>4</v>
       </c>
       <c r="B61" s="28" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C61" s="23"/>
       <c r="D61" s="24"/>
       <c r="E61" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F61" s="15" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G61" s="25" t="s">
         <v>49</v>
@@ -3409,15 +3380,15 @@
         <v>4</v>
       </c>
       <c r="B62" s="28" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C62" s="23"/>
       <c r="D62" s="24"/>
       <c r="E62" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G62" s="25" t="s">
         <v>49</v>
@@ -3434,15 +3405,15 @@
         <v>4</v>
       </c>
       <c r="B63" s="28" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C63" s="23"/>
       <c r="D63" s="24"/>
       <c r="E63" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F63" s="15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G63" s="25" t="s">
         <v>49</v>
@@ -3459,15 +3430,15 @@
         <v>4</v>
       </c>
       <c r="B64" s="28" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C64" s="23"/>
       <c r="D64" s="24"/>
       <c r="E64" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G64" s="25" t="s">
         <v>49</v>
@@ -3484,15 +3455,15 @@
         <v>4</v>
       </c>
       <c r="B65" s="28" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C65" s="23"/>
       <c r="D65" s="24"/>
       <c r="E65" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F65" s="15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G65" s="25" t="s">
         <v>49</v>
@@ -3509,15 +3480,15 @@
         <v>4</v>
       </c>
       <c r="B66" s="28" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C66" s="23"/>
       <c r="D66" s="24"/>
       <c r="E66" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="G66" s="25" t="s">
         <v>49</v>
@@ -3534,15 +3505,15 @@
         <v>4</v>
       </c>
       <c r="B67" s="28" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C67" s="23"/>
       <c r="D67" s="24"/>
       <c r="E67" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F67" s="15" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G67" s="25" t="s">
         <v>49</v>
@@ -3559,15 +3530,15 @@
         <v>4</v>
       </c>
       <c r="B68" s="28" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C68" s="23"/>
       <c r="D68" s="24"/>
       <c r="E68" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="G68" s="25" t="s">
         <v>49</v>
@@ -3584,15 +3555,15 @@
         <v>4</v>
       </c>
       <c r="B69" s="28" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C69" s="23"/>
       <c r="D69" s="24"/>
       <c r="E69" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F69" s="15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G69" s="25" t="s">
         <v>49</v>
@@ -3604,12 +3575,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="19" t="s">
-        <v>156</v>
-      </c>
+    <row r="70" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="19"/>
       <c r="B70" s="20" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C70" s="20"/>
       <c r="D70" s="20"/>
@@ -3624,15 +3593,15 @@
         <v>5</v>
       </c>
       <c r="B71" s="28" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C71" s="23"/>
       <c r="D71" s="24"/>
       <c r="E71" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F71" s="15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G71" s="25" t="s">
         <v>49</v>
@@ -3649,15 +3618,15 @@
         <v>5</v>
       </c>
       <c r="B72" s="28" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C72" s="23"/>
       <c r="D72" s="24"/>
       <c r="E72" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="G72" s="25" t="s">
         <v>49</v>
@@ -3674,15 +3643,15 @@
         <v>5</v>
       </c>
       <c r="B73" s="28" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C73" s="23"/>
       <c r="D73" s="24"/>
       <c r="E73" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F73" s="15" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="G73" s="25" t="s">
         <v>49</v>
@@ -3699,15 +3668,15 @@
         <v>5</v>
       </c>
       <c r="B74" s="28" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C74" s="23"/>
       <c r="D74" s="24"/>
       <c r="E74" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G74" s="25" t="s">
         <v>49</v>
@@ -3724,15 +3693,15 @@
         <v>5</v>
       </c>
       <c r="B75" s="28" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C75" s="23"/>
       <c r="D75" s="24"/>
       <c r="E75" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G75" s="25" t="s">
         <v>49</v>
@@ -3749,15 +3718,15 @@
         <v>5</v>
       </c>
       <c r="B76" s="28" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C76" s="23"/>
       <c r="D76" s="24"/>
       <c r="E76" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="G76" s="25" t="s">
         <v>49</v>
@@ -3774,15 +3743,15 @@
         <v>5</v>
       </c>
       <c r="B77" s="28" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C77" s="23"/>
       <c r="D77" s="24"/>
       <c r="E77" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F77" s="15" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G77" s="25" t="s">
         <v>49</v>
@@ -3799,15 +3768,15 @@
         <v>5</v>
       </c>
       <c r="B78" s="28" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C78" s="23"/>
       <c r="D78" s="24"/>
       <c r="E78" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F78" s="15" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G78" s="25" t="s">
         <v>49</v>
@@ -3824,15 +3793,15 @@
         <v>5</v>
       </c>
       <c r="B79" s="28" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C79" s="23"/>
       <c r="D79" s="24"/>
       <c r="E79" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G79" s="25" t="s">
         <v>49</v>
@@ -3849,15 +3818,15 @@
         <v>5</v>
       </c>
       <c r="B80" s="28" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C80" s="23"/>
       <c r="D80" s="24"/>
       <c r="E80" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F80" s="15" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G80" s="25" t="s">
         <v>49</v>
@@ -3874,15 +3843,15 @@
         <v>5</v>
       </c>
       <c r="B81" s="28" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C81" s="23"/>
       <c r="D81" s="24"/>
       <c r="E81" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F81" s="15" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G81" s="25" t="s">
         <v>49</v>
@@ -3899,15 +3868,15 @@
         <v>5</v>
       </c>
       <c r="B82" s="28" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C82" s="23"/>
       <c r="D82" s="24"/>
       <c r="E82" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="G82" s="25" t="s">
         <v>49</v>
@@ -3924,15 +3893,15 @@
         <v>5</v>
       </c>
       <c r="B83" s="28" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C83" s="23"/>
       <c r="D83" s="24"/>
       <c r="E83" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G83" s="25" t="s">
         <v>49</v>
@@ -3944,12 +3913,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="19" t="s">
-        <v>179</v>
-      </c>
+    <row r="84" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="19"/>
       <c r="B84" s="20" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C84" s="20"/>
       <c r="D84" s="20"/>
@@ -3964,15 +3931,15 @@
         <v>6</v>
       </c>
       <c r="B85" s="30" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C85" s="23"/>
       <c r="D85" s="24"/>
       <c r="E85" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F85" s="15" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="G85" s="25" t="s">
         <v>49</v>
@@ -3989,12 +3956,12 @@
         <v>6</v>
       </c>
       <c r="B86" s="30" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C86" s="23"/>
       <c r="D86" s="24"/>
       <c r="E86" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F86" s="15" t="s">
         <v>45</v>
@@ -4014,15 +3981,15 @@
         <v>6</v>
       </c>
       <c r="B87" s="30" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C87" s="23"/>
       <c r="D87" s="24"/>
       <c r="E87" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F87" s="15" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G87" s="25" t="s">
         <v>49</v>
@@ -4039,15 +4006,15 @@
         <v>6</v>
       </c>
       <c r="B88" s="30" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C88" s="23"/>
       <c r="D88" s="24"/>
       <c r="E88" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F88" s="15" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="G88" s="25" t="s">
         <v>49</v>
@@ -4064,15 +4031,15 @@
         <v>6</v>
       </c>
       <c r="B89" s="30" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C89" s="23"/>
       <c r="D89" s="24"/>
       <c r="E89" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F89" s="15" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="G89" s="25" t="s">
         <v>49</v>
@@ -4089,15 +4056,15 @@
         <v>6</v>
       </c>
       <c r="B90" s="30" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C90" s="23"/>
       <c r="D90" s="24"/>
       <c r="E90" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F90" s="15" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="G90" s="25" t="s">
         <v>49</v>
@@ -4114,15 +4081,15 @@
         <v>6</v>
       </c>
       <c r="B91" s="30" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C91" s="23"/>
       <c r="D91" s="24"/>
       <c r="E91" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F91" s="15" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="G91" s="25" t="s">
         <v>49</v>
@@ -4139,15 +4106,15 @@
         <v>6</v>
       </c>
       <c r="B92" s="30" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C92" s="23"/>
       <c r="D92" s="24"/>
       <c r="E92" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F92" s="15" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="G92" s="25" t="s">
         <v>49</v>
@@ -4164,15 +4131,15 @@
         <v>6</v>
       </c>
       <c r="B93" s="30" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C93" s="23"/>
       <c r="D93" s="24"/>
       <c r="E93" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F93" s="15" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G93" s="25" t="s">
         <v>49</v>
@@ -4189,15 +4156,15 @@
         <v>6</v>
       </c>
       <c r="B94" s="30" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C94" s="23"/>
       <c r="D94" s="24"/>
       <c r="E94" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F94" s="15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G94" s="25" t="s">
         <v>49</v>
@@ -4214,15 +4181,15 @@
         <v>6</v>
       </c>
       <c r="B95" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C95" s="23"/>
       <c r="D95" s="24"/>
       <c r="E95" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F95" s="15" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="G95" s="25" t="s">
         <v>49</v>
@@ -4239,15 +4206,15 @@
         <v>6</v>
       </c>
       <c r="B96" s="30" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C96" s="23"/>
       <c r="D96" s="24"/>
       <c r="E96" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F96" s="15" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="G96" s="25" t="s">
         <v>49</v>
@@ -4264,15 +4231,15 @@
         <v>6</v>
       </c>
       <c r="B97" s="30" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C97" s="23"/>
       <c r="D97" s="24"/>
       <c r="E97" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F97" s="15" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G97" s="25" t="s">
         <v>49</v>
@@ -4289,15 +4256,15 @@
         <v>6</v>
       </c>
       <c r="B98" s="30" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C98" s="23"/>
       <c r="D98" s="24"/>
       <c r="E98" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F98" s="15" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="G98" s="25" t="s">
         <v>49</v>
@@ -4314,15 +4281,15 @@
         <v>6</v>
       </c>
       <c r="B99" s="30" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C99" s="23"/>
       <c r="D99" s="24"/>
       <c r="E99" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F99" s="15" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G99" s="25" t="s">
         <v>49</v>
@@ -4339,15 +4306,15 @@
         <v>6</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C100" s="23"/>
       <c r="D100" s="24"/>
       <c r="E100" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F100" s="15" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="G100" s="25" t="s">
         <v>49</v>
@@ -4364,15 +4331,15 @@
         <v>6</v>
       </c>
       <c r="B101" s="30" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C101" s="23"/>
       <c r="D101" s="24"/>
       <c r="E101" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F101" s="15" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="G101" s="25" t="s">
         <v>49</v>
@@ -4384,12 +4351,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="19" t="s">
-        <v>209</v>
-      </c>
+    <row r="102" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="19"/>
       <c r="B102" s="20" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C102" s="20"/>
       <c r="D102" s="20"/>
@@ -4404,15 +4369,15 @@
         <v>7</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C103" s="23"/>
       <c r="D103" s="24"/>
       <c r="E103" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F103" s="15" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="G103" s="25" t="s">
         <v>49</v>
@@ -4429,15 +4394,15 @@
         <v>7</v>
       </c>
       <c r="B104" s="32" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C104" s="23"/>
       <c r="D104" s="24"/>
       <c r="E104" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F104" s="15" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G104" s="25" t="s">
         <v>49</v>
@@ -4454,15 +4419,15 @@
         <v>7</v>
       </c>
       <c r="B105" s="32" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C105" s="23"/>
       <c r="D105" s="24"/>
       <c r="E105" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F105" s="15" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G105" s="25" t="s">
         <v>49</v>
@@ -4479,15 +4444,15 @@
         <v>7</v>
       </c>
       <c r="B106" s="32" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C106" s="23"/>
       <c r="D106" s="24"/>
       <c r="E106" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F106" s="15" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="G106" s="25" t="s">
         <v>49</v>
@@ -4504,15 +4469,15 @@
         <v>7</v>
       </c>
       <c r="B107" s="32" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C107" s="23"/>
       <c r="D107" s="24"/>
       <c r="E107" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F107" s="15" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G107" s="25" t="s">
         <v>49</v>
@@ -4529,15 +4494,15 @@
         <v>7</v>
       </c>
       <c r="B108" s="32" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="C108" s="23"/>
       <c r="D108" s="24"/>
       <c r="E108" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F108" s="15" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="G108" s="25" t="s">
         <v>49</v>
@@ -4554,15 +4519,15 @@
         <v>7</v>
       </c>
       <c r="B109" s="32" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C109" s="23"/>
       <c r="D109" s="24"/>
       <c r="E109" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F109" s="15" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G109" s="25" t="s">
         <v>49</v>
@@ -4579,15 +4544,15 @@
         <v>7</v>
       </c>
       <c r="B110" s="32" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C110" s="23"/>
       <c r="D110" s="24"/>
       <c r="E110" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F110" s="15" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="G110" s="25" t="s">
         <v>49</v>
@@ -4604,15 +4569,15 @@
         <v>7</v>
       </c>
       <c r="B111" s="32" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C111" s="23"/>
       <c r="D111" s="24"/>
       <c r="E111" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F111" s="15" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="G111" s="25" t="s">
         <v>49</v>
@@ -4629,15 +4594,15 @@
         <v>7</v>
       </c>
       <c r="B112" s="32" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C112" s="23"/>
       <c r="D112" s="24"/>
       <c r="E112" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F112" s="15" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="G112" s="25" t="s">
         <v>49</v>
@@ -4654,15 +4619,15 @@
         <v>7</v>
       </c>
       <c r="B113" s="32" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C113" s="23"/>
       <c r="D113" s="24"/>
       <c r="E113" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F113" s="15" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="G113" s="25" t="s">
         <v>49</v>
@@ -4679,15 +4644,15 @@
         <v>7</v>
       </c>
       <c r="B114" s="32" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C114" s="23"/>
       <c r="D114" s="24"/>
       <c r="E114" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F114" s="15" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="G114" s="25" t="s">
         <v>49</v>
@@ -4704,15 +4669,15 @@
         <v>7</v>
       </c>
       <c r="B115" s="32" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C115" s="23"/>
       <c r="D115" s="24"/>
       <c r="E115" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F115" s="15" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="G115" s="25" t="s">
         <v>49</v>
@@ -4729,15 +4694,15 @@
         <v>7</v>
       </c>
       <c r="B116" s="32" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C116" s="23"/>
       <c r="D116" s="24"/>
       <c r="E116" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F116" s="15" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="G116" s="25" t="s">
         <v>49</v>
@@ -4754,15 +4719,15 @@
         <v>7</v>
       </c>
       <c r="B117" s="32" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C117" s="23"/>
       <c r="D117" s="24"/>
       <c r="E117" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F117" s="15" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="G117" s="25" t="s">
         <v>49</v>
@@ -4774,12 +4739,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="19" t="s">
-        <v>228</v>
-      </c>
+    <row r="118" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="19"/>
       <c r="B118" s="20" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="C118" s="20"/>
       <c r="D118" s="20"/>
@@ -4794,15 +4757,15 @@
         <v>8</v>
       </c>
       <c r="B119" s="32" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C119" s="23"/>
       <c r="D119" s="24"/>
       <c r="E119" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F119" s="15" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G119" s="25" t="s">
         <v>49</v>
@@ -4819,15 +4782,15 @@
         <v>8</v>
       </c>
       <c r="B120" s="32" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C120" s="23"/>
       <c r="D120" s="24"/>
       <c r="E120" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F120" s="15" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="G120" s="25" t="s">
         <v>49</v>
@@ -4844,15 +4807,15 @@
         <v>8</v>
       </c>
       <c r="B121" s="32" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C121" s="23"/>
       <c r="D121" s="24"/>
       <c r="E121" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F121" s="15" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G121" s="25" t="s">
         <v>49</v>
@@ -4869,15 +4832,15 @@
         <v>8</v>
       </c>
       <c r="B122" s="32" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C122" s="23"/>
       <c r="D122" s="24"/>
       <c r="E122" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F122" s="15" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="G122" s="25" t="s">
         <v>49</v>
@@ -4894,15 +4857,15 @@
         <v>8</v>
       </c>
       <c r="B123" s="32" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C123" s="23"/>
       <c r="D123" s="24"/>
       <c r="E123" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F123" s="15" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="G123" s="25" t="s">
         <v>49</v>
@@ -4919,15 +4882,15 @@
         <v>8</v>
       </c>
       <c r="B124" s="32" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C124" s="23"/>
       <c r="D124" s="24"/>
       <c r="E124" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F124" s="15" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="G124" s="25" t="s">
         <v>49</v>
@@ -4944,15 +4907,15 @@
         <v>8</v>
       </c>
       <c r="B125" s="32" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C125" s="23"/>
       <c r="D125" s="24"/>
       <c r="E125" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F125" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G125" s="25" t="s">
         <v>49</v>
@@ -4969,15 +4932,15 @@
         <v>8</v>
       </c>
       <c r="B126" s="32" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C126" s="23"/>
       <c r="D126" s="24"/>
       <c r="E126" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F126" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G126" s="26"/>
       <c r="H126" s="26"/>
@@ -4988,15 +4951,15 @@
         <v>8</v>
       </c>
       <c r="B127" s="32" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C127" s="23"/>
       <c r="D127" s="24"/>
       <c r="E127" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F127" s="15" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="G127" s="25" t="s">
         <v>49</v>
@@ -5013,15 +4976,15 @@
         <v>8</v>
       </c>
       <c r="B128" s="32" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C128" s="23"/>
       <c r="D128" s="24"/>
       <c r="E128" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F128" s="15" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="G128" s="25" t="s">
         <v>49</v>

</xml_diff>